<commit_message>
clean contract bugs fixed, working through adobe script utils now
</commit_message>
<xml_diff>
--- a/010-npm_node/02-results/2108AC01S Tapestry (Discovery Phase III) REV 1x.xlsx
+++ b/010-npm_node/02-results/2108AC01S Tapestry (Discovery Phase III) REV 1x.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P199"/>
+  <dimension ref="A1:L198"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -437,18 +437,6 @@
       <c r="L1" t="str">
         <v>11</v>
       </c>
-      <c r="M1" t="str">
-        <v>12</v>
-      </c>
-      <c r="N1" t="str">
-        <v>13</v>
-      </c>
-      <c r="O1" t="str">
-        <v>14</v>
-      </c>
-      <c r="P1" t="str">
-        <v>15</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -487,18 +475,6 @@
       <c r="L2" t="str">
         <v>CONTRACT_FILE</v>
       </c>
-      <c r="M2" t="str">
-        <v>4</v>
-      </c>
-      <c r="N2" t="str">
-        <v>5</v>
-      </c>
-      <c r="O2" t="str">
-        <v>6</v>
-      </c>
-      <c r="P2" t="str">
-        <v>8</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -7876,26 +7852,38 @@
       <c r="A197" t="str">
         <v xml:space="preserve">#17: AMENITY SIGNAGE </v>
       </c>
-      <c r="E197" t="str">
-        <v>2108AC01S</v>
-      </c>
-      <c r="F197" t="str">
-        <v>TAPESTRY (DISCOVERY PHASE III)</v>
+      <c r="B197" t="str">
+        <v>I.</v>
+      </c>
+      <c r="C197">
+        <v>1</v>
+      </c>
+      <c r="D197" t="str">
+        <v>DOG PARK ID / POLICY - FENCE MOUNT</v>
+      </c>
+      <c r="E197">
+        <v>595</v>
+      </c>
+      <c r="F197">
+        <v>595</v>
       </c>
       <c r="G197" t="str">
-        <v>2108AC01S Tapestry (Discovery Phase III) REV 1x.xlsx</v>
-      </c>
-      <c r="M197" t="str">
-        <v xml:space="preserve"> X1 @ SMALL POOL)</v>
-      </c>
-      <c r="N197" t="str">
-        <v>ANDRES CONSTRUCTION SERVICES LLC (Construction Manager / General Contractor) 3710 Rawlins Street Suite 1510 |  Dallas, Texas 75219</v>
-      </c>
-      <c r="O197" t="str">
-        <v>Kyle Washington (Project manager)</v>
-      </c>
-      <c r="P197" t="str">
-        <v>09.23.21 01.19.23 REV 1</v>
+        <v>ANDRES CONSTRUCTION SERVICES LLC (Construction Manager / General Contractor) 3710 Rawlins Street Suite 1510 |  Dallas, Texas 75219</v>
+      </c>
+      <c r="H197" t="str">
+        <v>Kyle Washington (Project manager)</v>
+      </c>
+      <c r="I197" t="str">
+        <v>2108AC01S</v>
+      </c>
+      <c r="J197" t="str">
+        <v>09.23.21 01.19.23 REV 1</v>
+      </c>
+      <c r="K197" t="str">
+        <v>TAPESTRY (DISCOVERY PHASE III)</v>
+      </c>
+      <c r="L197" t="str">
+        <v>2108AC01S Tapestry (Discovery Phase III) REV 1x.xlsx</v>
       </c>
     </row>
     <row r="198">
@@ -7903,19 +7891,19 @@
         <v xml:space="preserve">#17: AMENITY SIGNAGE </v>
       </c>
       <c r="B198" t="str">
-        <v>I.</v>
+        <v>J.</v>
       </c>
       <c r="C198">
         <v>1</v>
       </c>
       <c r="D198" t="str">
-        <v>DOG PARK ID / POLICY - FENCE MOUNT</v>
+        <v>FIRE PIT GUIDELINES PLAQUE</v>
       </c>
       <c r="E198">
-        <v>595</v>
+        <v>110</v>
       </c>
       <c r="F198">
-        <v>595</v>
+        <v>110</v>
       </c>
       <c r="G198" t="str">
         <v>ANDRES CONSTRUCTION SERVICES LLC (Construction Manager / General Contractor) 3710 Rawlins Street Suite 1510 |  Dallas, Texas 75219</v>
@@ -7933,50 +7921,12 @@
         <v>TAPESTRY (DISCOVERY PHASE III)</v>
       </c>
       <c r="L198" t="str">
-        <v>2108AC01S Tapestry (Discovery Phase III) REV 1x.xlsx</v>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" t="str">
-        <v xml:space="preserve">#17: AMENITY SIGNAGE </v>
-      </c>
-      <c r="B199" t="str">
-        <v>J.</v>
-      </c>
-      <c r="C199">
-        <v>1</v>
-      </c>
-      <c r="D199" t="str">
-        <v>FIRE PIT GUIDELINES PLAQUE</v>
-      </c>
-      <c r="E199">
-        <v>110</v>
-      </c>
-      <c r="F199">
-        <v>110</v>
-      </c>
-      <c r="G199" t="str">
-        <v>ANDRES CONSTRUCTION SERVICES LLC (Construction Manager / General Contractor) 3710 Rawlins Street Suite 1510 |  Dallas, Texas 75219</v>
-      </c>
-      <c r="H199" t="str">
-        <v>Kyle Washington (Project manager)</v>
-      </c>
-      <c r="I199" t="str">
-        <v>2108AC01S</v>
-      </c>
-      <c r="J199" t="str">
-        <v>09.23.21 01.19.23 REV 1</v>
-      </c>
-      <c r="K199" t="str">
-        <v>TAPESTRY (DISCOVERY PHASE III)</v>
-      </c>
-      <c r="L199" t="str">
         <v>2108AC01S Tapestry (Discovery Phase III) REV 1x.xlsx</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P199"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L198"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>